<commit_message>
Port 4.0.7 transportation inputs from main into develop
- Travel: BCDTRtSY and BAADTbVT rebased to AEO 2026 as on main (passenger-LDV
  miles per vehicle 10,411 in 2024); develop's seam fix removed, boat activity kept.
- ZEV requirement: main's BRZSPbS/RZSPbS (ACC I credit 0.08 through 2025, 0 after).
- TTS: on-road shareweights recalibrated on develop to main's AEO 2026 shares
  (eps-calibrate step 3a, 3 passes; 2025 passenger-LDV BEV 5.07% vs 5.05% observed),
  main's PHEV 2050 targets, main's calibration records; motorbikes re-exported.
- Small fixes from main: RTMF workbook column, SoVCaPC, FpUCD header, BRASC precision.
</commit_message>
<xml_diff>
--- a/InputData/trans/RTMF/Recipient Transportation Mode Fractions.xlsx
+++ b/InputData/trans/RTMF/Recipient Transportation Mode Fractions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\RTMF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2643F14-5F7F-4432-8B4A-9A19F1481256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E945319C-3F0F-4E25-85D1-D5C5DF30BEF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,6 +29,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -666,15 +668,14 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" customWidth="1"/>
     <col min="7" max="7" width="11.5703125" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -696,11 +697,11 @@
       <c r="G1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -722,12 +723,12 @@
       <c r="G2">
         <v>0</v>
       </c>
-      <c r="I2" s="4">
+      <c r="H2" s="4">
         <f>1-SUM(B2:G2)</f>
         <v>0.33999999999999997</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -749,12 +750,12 @@
       <c r="G3">
         <v>0</v>
       </c>
-      <c r="I3" s="4">
-        <f t="shared" ref="I3:I7" si="0">1-SUM(B3:G3)</f>
+      <c r="H3" s="4">
+        <f t="shared" ref="H3:H7" si="0">1-SUM(B3:G3)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -776,12 +777,12 @@
       <c r="G4">
         <v>0</v>
       </c>
-      <c r="I4" s="4">
+      <c r="H4" s="4">
         <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -803,12 +804,12 @@
       <c r="G5">
         <v>0</v>
       </c>
-      <c r="I5" s="4">
+      <c r="H5" s="4">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -830,12 +831,12 @@
       <c r="G6">
         <v>0</v>
       </c>
-      <c r="I6" s="4">
+      <c r="H6" s="4">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -857,7 +858,7 @@
       <c r="G7">
         <v>0</v>
       </c>
-      <c r="I7" s="4">
+      <c r="H7" s="4">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -872,15 +873,14 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" customWidth="1"/>
     <col min="7" max="7" width="11.5703125" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -902,11 +902,11 @@
       <c r="G1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -928,12 +928,12 @@
       <c r="G2">
         <v>0</v>
       </c>
-      <c r="I2" s="4">
+      <c r="H2" s="4">
         <f>1-SUM(B2:G2)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -955,12 +955,12 @@
       <c r="G3">
         <v>0</v>
       </c>
-      <c r="I3" s="4">
-        <f t="shared" ref="I3:I7" si="0">1-SUM(B3:G3)</f>
+      <c r="H3" s="4">
+        <f t="shared" ref="H3:H7" si="0">1-SUM(B3:G3)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -982,12 +982,12 @@
       <c r="G4">
         <v>0</v>
       </c>
-      <c r="I4" s="4">
+      <c r="H4" s="4">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -1009,12 +1009,12 @@
       <c r="G5">
         <v>0</v>
       </c>
-      <c r="I5" s="4">
+      <c r="H5" s="4">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -1036,12 +1036,12 @@
       <c r="G6">
         <v>0</v>
       </c>
-      <c r="I6" s="4">
+      <c r="H6" s="4">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1063,7 +1063,7 @@
       <c r="G7">
         <v>0</v>
       </c>
-      <c r="I7" s="4">
+      <c r="H7" s="4">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>

</xml_diff>